<commit_message>
Relax teacher import class assignment requirements
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
+++ b/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
   <si>
     <t>ad</t>
   </si>
@@ -23,12 +23,6 @@
     <t>brans</t>
   </si>
   <si>
-    <t>atanacak_sinif</t>
-  </si>
-  <si>
-    <t>ders</t>
-  </si>
-  <si>
     <t>tc_kimlik_no</t>
   </si>
   <si>
@@ -44,9 +38,6 @@
     <t>Matematik</t>
   </si>
   <si>
-    <t>8-A</t>
-  </si>
-  <si>
     <t>10000001440</t>
   </si>
   <si>
@@ -71,9 +62,6 @@
     <t>Fen Bilimleri</t>
   </si>
   <si>
-    <t>8-B</t>
-  </si>
-  <si>
     <t>10000001686</t>
   </si>
   <si>
@@ -86,19 +74,13 @@
     <t>Kabul edilen değerler</t>
   </si>
   <si>
-    <t>Uygulamadaki sınıf adıyla aynı olmalı. Örnek: 8-A, 8-B, 10-A</t>
-  </si>
-  <si>
-    <t>Uygulamadaki ders adıyla aynı olmalı. Örnek: Matematik, Türkçe, Fen Bilimleri</t>
+    <t>Öğretmenin branşı. Sınıf ve ders atamaları uygulamada öğretmen detayından yapılır.</t>
   </si>
   <si>
     <t>Öğretmen portal hesabı açılacaksa 11 haneli TC kimlik no. Telefonla birlikte doldurun veya ikisini de boş bırakın.</t>
   </si>
   <si>
     <t>Öğretmen portal hesabı açılacaksa telefon. TC kimlik no ile birlikte doldurun veya ikisini de boş bırakın.</t>
-  </si>
-  <si>
-    <t>Öğretmenin branşı. Ders kolonu boşsa eski şablon uyumluluğu için branş ders olarak denenir.</t>
   </si>
 </sst>
 </file>
@@ -195,32 +177,28 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="OgretmenAktarimTablosu" displayName="OgretmenAktarimTablosu" ref="A1:G4" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A1:G4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="OgretmenAktarimTablosu" displayName="OgretmenAktarimTablosu" ref="A1:E4" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A1:E4">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
     <filterColumn colId="3" hiddenButton="1"/>
     <filterColumn colId="4" hiddenButton="1"/>
-    <filterColumn colId="5" hiddenButton="1"/>
-    <filterColumn colId="6" hiddenButton="1"/>
   </autoFilter>
-  <tableColumns count="7">
+  <tableColumns count="5">
     <tableColumn id="1" name="ad" totalsRowLabel="Total"/>
     <tableColumn id="2" name="soyad" totalsRowFunction="none"/>
     <tableColumn id="3" name="brans" totalsRowFunction="none"/>
-    <tableColumn id="4" name="atanacak_sinif" totalsRowFunction="none"/>
-    <tableColumn id="5" name="ders" totalsRowFunction="none"/>
-    <tableColumn id="6" name="tc_kimlik_no" totalsRowFunction="none"/>
-    <tableColumn id="7" name="telefon" totalsRowFunction="none"/>
+    <tableColumn id="4" name="tc_kimlik_no" totalsRowFunction="none"/>
+    <tableColumn id="5" name="telefon" totalsRowFunction="none"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" name="OgretmenSecenekleri" displayName="OgretmenSecenekleri" ref="A1:B6" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A1:B6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" name="OgretmenSecenekleri" displayName="OgretmenSecenekleri" ref="A1:B4" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A1:B4">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
@@ -554,18 +532,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -581,80 +557,56 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>10</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="B4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -668,7 +620,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -677,50 +629,34 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix teacher import template tc values
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
+++ b/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
@@ -74,7 +74,7 @@
     <t>İngilizce</t>
   </si>
   <si>
-    <t>10000001687</t>
+    <t>10000001754</t>
   </si>
   <si>
     <t>5550000017</t>
@@ -86,7 +86,7 @@
     <t>Sosyal Bilimler</t>
   </si>
   <si>
-    <t>10000001688</t>
+    <t>10000001822</t>
   </si>
   <si>
     <t>5550000018</t>
@@ -95,7 +95,7 @@
     <t>Merve</t>
   </si>
   <si>
-    <t>10000001689</t>
+    <t>10000001990</t>
   </si>
   <si>
     <t>5550000019</t>
@@ -104,7 +104,7 @@
     <t>Osman</t>
   </si>
   <si>
-    <t>10000001690</t>
+    <t>10000002058</t>
   </si>
   <si>
     <t>5550000020</t>
@@ -113,7 +113,7 @@
     <t>Tuğba</t>
   </si>
   <si>
-    <t>10000001691</t>
+    <t>10000002126</t>
   </si>
   <si>
     <t>5550000021</t>
@@ -122,7 +122,7 @@
     <t>Mustafa</t>
   </si>
   <si>
-    <t>10000001692</t>
+    <t>10000002294</t>
   </si>
   <si>
     <t>5550000022</t>
@@ -134,7 +134,7 @@
     <t>Din Kültürü ve Ahlak Bilgisi</t>
   </si>
   <si>
-    <t>10000001693</t>
+    <t>10000002362</t>
   </si>
   <si>
     <t>5550000023</t>
@@ -143,7 +143,7 @@
     <t>Melike</t>
   </si>
   <si>
-    <t>10000001694</t>
+    <t>10000002430</t>
   </si>
   <si>
     <t>5550000024</t>
@@ -764,7 +764,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -811,6 +811,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove redundant teacher template course column
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
+++ b/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
   <si>
     <t>ad</t>
   </si>
@@ -33,31 +33,31 @@
     <t>atanacak_sinif</t>
   </si>
   <si>
+    <t>alan</t>
+  </si>
+  <si>
+    <t>aciklama</t>
+  </si>
+  <si>
+    <t>Ogretmen adi. Zorunludur.</t>
+  </si>
+  <si>
+    <t>Ogretmen soyadi. Zorunludur.</t>
+  </si>
+  <si>
+    <t>Ogretmenin ana bransi. Bos birakilabilir.</t>
+  </si>
+  <si>
+    <t>Ogretmen TC kimlik no. Bos birakilabilir; doluysa 11 haneli ve gecerli olmalidir.</t>
+  </si>
+  <si>
+    <t>Ogretmen cep telefonu. Bos birakilabilir.</t>
+  </si>
+  <si>
+    <t>Ogretmenin atanacagi sinif adi. Bos birakilabilir.</t>
+  </si>
+  <si>
     <t>ders</t>
-  </si>
-  <si>
-    <t>alan</t>
-  </si>
-  <si>
-    <t>aciklama</t>
-  </si>
-  <si>
-    <t>Ogretmen adi. Zorunludur.</t>
-  </si>
-  <si>
-    <t>Ogretmen soyadi. Zorunludur.</t>
-  </si>
-  <si>
-    <t>Ogretmenin ana bransi. Bos birakilabilir.</t>
-  </si>
-  <si>
-    <t>Ogretmen TC kimlik no. Bos birakilabilir; doluysa 11 haneli ve gecerli olmalidir.</t>
-  </si>
-  <si>
-    <t>Ogretmen cep telefonu. Bos birakilabilir.</t>
-  </si>
-  <si>
-    <t>Ogretmenin atanacagi sinif adi. Bos birakilabilir.</t>
   </si>
   <si>
     <t>Atanacak sinifta okutacagi ders adi. Bos birakilabilir.</t>
@@ -474,7 +474,6 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -495,9 +494,6 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -518,10 +514,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -529,7 +525,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -537,7 +533,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -545,7 +541,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -553,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -561,7 +557,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -569,12 +565,12 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
@@ -597,7 +593,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>16</v>
@@ -637,7 +633,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Remove redundant teacher template course column (#29)
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
+++ b/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
   <si>
     <t>ad</t>
   </si>
@@ -33,31 +33,31 @@
     <t>atanacak_sinif</t>
   </si>
   <si>
+    <t>alan</t>
+  </si>
+  <si>
+    <t>aciklama</t>
+  </si>
+  <si>
+    <t>Ogretmen adi. Zorunludur.</t>
+  </si>
+  <si>
+    <t>Ogretmen soyadi. Zorunludur.</t>
+  </si>
+  <si>
+    <t>Ogretmenin ana bransi. Bos birakilabilir.</t>
+  </si>
+  <si>
+    <t>Ogretmen TC kimlik no. Bos birakilabilir; doluysa 11 haneli ve gecerli olmalidir.</t>
+  </si>
+  <si>
+    <t>Ogretmen cep telefonu. Bos birakilabilir.</t>
+  </si>
+  <si>
+    <t>Ogretmenin atanacagi sinif adi. Bos birakilabilir.</t>
+  </si>
+  <si>
     <t>ders</t>
-  </si>
-  <si>
-    <t>alan</t>
-  </si>
-  <si>
-    <t>aciklama</t>
-  </si>
-  <si>
-    <t>Ogretmen adi. Zorunludur.</t>
-  </si>
-  <si>
-    <t>Ogretmen soyadi. Zorunludur.</t>
-  </si>
-  <si>
-    <t>Ogretmenin ana bransi. Bos birakilabilir.</t>
-  </si>
-  <si>
-    <t>Ogretmen TC kimlik no. Bos birakilabilir; doluysa 11 haneli ve gecerli olmalidir.</t>
-  </si>
-  <si>
-    <t>Ogretmen cep telefonu. Bos birakilabilir.</t>
-  </si>
-  <si>
-    <t>Ogretmenin atanacagi sinif adi. Bos birakilabilir.</t>
   </si>
   <si>
     <t>Atanacak sinifta okutacagi ders adi. Bos birakilabilir.</t>
@@ -474,7 +474,6 @@
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -495,9 +494,6 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -518,10 +514,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -529,7 +525,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -537,7 +533,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -545,7 +541,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -553,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -561,7 +557,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -569,12 +565,12 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
         <v>15</v>
@@ -597,7 +593,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>16</v>
@@ -637,7 +633,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="B6" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Remove teacher template class column
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
+++ b/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="22">
   <si>
     <t>ad</t>
   </si>
@@ -30,28 +30,28 @@
     <t>telefon</t>
   </si>
   <si>
+    <t>alan</t>
+  </si>
+  <si>
+    <t>aciklama</t>
+  </si>
+  <si>
+    <t>Ogretmen adi. Zorunludur.</t>
+  </si>
+  <si>
+    <t>Ogretmen soyadi. Zorunludur.</t>
+  </si>
+  <si>
+    <t>Ogretmenin ana bransi. Bos birakilabilir.</t>
+  </si>
+  <si>
+    <t>Ogretmen TC kimlik no. Bos birakilabilir; doluysa 11 haneli ve gecerli olmalidir.</t>
+  </si>
+  <si>
+    <t>Ogretmen cep telefonu. Bos birakilabilir.</t>
+  </si>
+  <si>
     <t>atanacak_sinif</t>
-  </si>
-  <si>
-    <t>alan</t>
-  </si>
-  <si>
-    <t>aciklama</t>
-  </si>
-  <si>
-    <t>Ogretmen adi. Zorunludur.</t>
-  </si>
-  <si>
-    <t>Ogretmen soyadi. Zorunludur.</t>
-  </si>
-  <si>
-    <t>Ogretmenin ana bransi. Bos birakilabilir.</t>
-  </si>
-  <si>
-    <t>Ogretmen TC kimlik no. Bos birakilabilir; doluysa 11 haneli ve gecerli olmalidir.</t>
-  </si>
-  <si>
-    <t>Ogretmen cep telefonu. Bos birakilabilir.</t>
   </si>
   <si>
     <t>Ogretmenin atanacagi sinif adi. Bos birakilabilir.</t>
@@ -467,16 +467,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -491,9 +490,6 @@
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -514,10 +510,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -525,7 +521,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -533,7 +529,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -541,7 +537,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -549,7 +545,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -557,12 +553,12 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
         <v>13</v>
@@ -593,7 +589,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>16</v>
@@ -625,7 +621,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
Remove teacher template class column (#30)
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
+++ b/apps/web/public/templates/ogretmen-aktarim-sablonu.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="22">
   <si>
     <t>ad</t>
   </si>
@@ -30,28 +30,28 @@
     <t>telefon</t>
   </si>
   <si>
+    <t>alan</t>
+  </si>
+  <si>
+    <t>aciklama</t>
+  </si>
+  <si>
+    <t>Ogretmen adi. Zorunludur.</t>
+  </si>
+  <si>
+    <t>Ogretmen soyadi. Zorunludur.</t>
+  </si>
+  <si>
+    <t>Ogretmenin ana bransi. Bos birakilabilir.</t>
+  </si>
+  <si>
+    <t>Ogretmen TC kimlik no. Bos birakilabilir; doluysa 11 haneli ve gecerli olmalidir.</t>
+  </si>
+  <si>
+    <t>Ogretmen cep telefonu. Bos birakilabilir.</t>
+  </si>
+  <si>
     <t>atanacak_sinif</t>
-  </si>
-  <si>
-    <t>alan</t>
-  </si>
-  <si>
-    <t>aciklama</t>
-  </si>
-  <si>
-    <t>Ogretmen adi. Zorunludur.</t>
-  </si>
-  <si>
-    <t>Ogretmen soyadi. Zorunludur.</t>
-  </si>
-  <si>
-    <t>Ogretmenin ana bransi. Bos birakilabilir.</t>
-  </si>
-  <si>
-    <t>Ogretmen TC kimlik no. Bos birakilabilir; doluysa 11 haneli ve gecerli olmalidir.</t>
-  </si>
-  <si>
-    <t>Ogretmen cep telefonu. Bos birakilabilir.</t>
   </si>
   <si>
     <t>Ogretmenin atanacagi sinif adi. Bos birakilabilir.</t>
@@ -467,16 +467,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="14" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -491,9 +490,6 @@
       </c>
       <c r="E1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -514,10 +510,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -525,7 +521,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -533,7 +529,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -541,7 +537,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -549,7 +545,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -557,12 +553,12 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B7" t="s">
         <v>13</v>
@@ -593,7 +589,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>16</v>
@@ -625,7 +621,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>

</xml_diff>